<commit_message>
Update sheriff sale 2026-11-02 (list printed 10/22/2026 2:51PM)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KpGKyBZFowribbp2E9FYwu
</commit_message>
<xml_diff>
--- a/state/2026-11-02.xlsx
+++ b/state/2026-11-02.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM).  Updated Sun Oct 25, 2026 10:15 PM.</t>
+          <t>Source: November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM).  Updated Mon Oct 26, 2026 4:31 AM.</t>
         </is>
       </c>
     </row>
@@ -605,14 +605,14 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Changes since the last update</t>
+          <t>Changes since the last update (2026-10-25 22:15)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>First version for this auction — future updates will list what changed here.</t>
+          <t>No changes to OK to Sell or Almost Ready.</t>
         </is>
       </c>
     </row>
@@ -663,8 +663,26 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:31</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>105</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" ht="48" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>How to use: type only in the yellow YOUR ENTRY columns on OK to Sell / Almost Ready (assessed value fills in the transfer-tax estimate). Every update keeps what you typed, matched by Sale ID. The Sheriff finalizes the list the morning of the sale — check the morning-of list before bidding. Not legal advice; see Glossary.</t>
         </is>
@@ -672,7 +690,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40169,7 +40187,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40204,7 +40222,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-25 22:15</t>
+          <t>2026-10-26 04:31</t>
         </is>
       </c>
     </row>
@@ -40228,6 +40246,29 @@
         </is>
       </c>
       <c r="E4" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-10-26 04:31</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>105</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM)</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>17</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update sheriff sale 2026-11-02 (list printed 10/22/2026 2:51PM, no changes)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VqwE5GftwuqMUQXhJbGRx2
</commit_message>
<xml_diff>
--- a/state/2026-11-02.xlsx
+++ b/state/2026-11-02.xlsx
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -548,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Source: November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM).  Updated Mon Oct 26, 2026 4:31 AM.</t>
+          <t>Source: November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM).  Updated Wed Oct 28, 2026 4:31 AM.</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Changes since the last update (2026-10-25 22:15)</t>
+          <t>Changes since the last update (2026-10-26 04:31)</t>
         </is>
       </c>
     </row>
@@ -681,8 +681,26 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-28 04:31</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>105</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>How to use: type only in the yellow YOUR ENTRY columns on OK to Sell / Almost Ready (assessed value fills in the transfer-tax estimate). Every update keeps what you typed, matched by Sale ID. The Sheriff finalizes the list the morning of the sale — check the morning-of list before bidding. Not legal advice; see Glossary.</t>
         </is>
@@ -690,7 +708,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40187,7 +40205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -40222,7 +40240,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-26 04:31</t>
+          <t>2026-10-28 04:31</t>
         </is>
       </c>
     </row>
@@ -40269,6 +40287,29 @@
         </is>
       </c>
       <c r="E5" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>log</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-10-28 04:31</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>105</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>November-Sale-List-Updated-10-22.pdf (printed 10/22/2026 2:51:38PM)</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>17</v>
       </c>
     </row>

</xml_diff>